<commit_message>
del almak because of new site structure
</commit_message>
<xml_diff>
--- a/outputs/analysiss.xlsx
+++ b/outputs/analysiss.xlsx
@@ -8,7 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="not in the list cars" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08-05-2024_@_17_56" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06-09-2024_@_14_43" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -478,7 +478,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Solaris SH</t>
+          <t>Solaris New 2024</t>
         </is>
       </c>
     </row>
@@ -488,7 +488,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Geely Belgee X50</t>
+          <t>Сhangan Alsvin</t>
         </is>
       </c>
     </row>
@@ -498,7 +498,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Haval Jolion 2WD</t>
+          <t>Solaris HS</t>
         </is>
       </c>
     </row>
@@ -508,7 +508,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Haval Jolion 4WD</t>
+          <t>Geely Belgee X50</t>
         </is>
       </c>
     </row>
@@ -518,7 +518,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Changan UNI-K</t>
+          <t>Haval Jolion 2WD</t>
         </is>
       </c>
     </row>
@@ -528,7 +528,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Geely Emgrand</t>
+          <t>Haval Jolion 4WD</t>
         </is>
       </c>
     </row>
@@ -538,7 +538,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Gac GS8 II</t>
+          <t>Haval F7X</t>
         </is>
       </c>
     </row>
@@ -548,7 +548,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Geely Atlas NEW Promo</t>
+          <t>Chery Tiggo 7 Pro Max</t>
         </is>
       </c>
     </row>
@@ -558,7 +558,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Geely Emgrand</t>
+          <t>Changan UNI-K</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Belgee X50</t>
+          <t>GAC M8</t>
         </is>
       </c>
     </row>
@@ -578,7 +578,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Hyundai Tucson IV AT</t>
+          <t>Geely Emgrand</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Geely Atlas NEW</t>
+          <t xml:space="preserve">Belgee X50 </t>
         </is>
       </c>
     </row>
@@ -598,7 +598,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Voyah Free</t>
+          <t>Gac GS3</t>
         </is>
       </c>
     </row>
@@ -608,7 +608,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Zeekr 001</t>
+          <t xml:space="preserve">Geely Preface </t>
         </is>
       </c>
     </row>
@@ -618,7 +618,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Zeekr 009</t>
+          <t>Geely Preface Flagship</t>
         </is>
       </c>
     </row>
@@ -628,7 +628,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Changan  UNI-K</t>
+          <t>Geely Atlas New 4 WD</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Changan CS 55 PLUS</t>
+          <t>Gac GS8 II</t>
         </is>
       </c>
     </row>
@@ -648,7 +648,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Changan UNI-T</t>
+          <t>Zeekr 009</t>
         </is>
       </c>
     </row>
@@ -658,7 +658,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Changan EADO</t>
+          <t>Changan  UNI-K</t>
         </is>
       </c>
     </row>
@@ -668,7 +668,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Jaguar XE ВК49865</t>
+          <t>Changan CS 55 PLUS</t>
         </is>
       </c>
     </row>
@@ -678,7 +678,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Zeekr 001</t>
+          <t>Changan UNI-T</t>
         </is>
       </c>
     </row>
@@ -687,6 +687,36 @@
         <v>21</v>
       </c>
       <c r="B23" t="inlineStr">
+        <is>
+          <t>Changan EADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="1" t="n">
+        <v>22</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Jaguar XE ВК49865</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="1" t="n">
+        <v>23</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Zeekr 001</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="1" t="n">
+        <v>24</v>
+      </c>
+      <c r="B26" t="inlineStr">
         <is>
           <t>Lixang Li 9</t>
         </is>
@@ -703,7 +733,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K155"/>
+  <dimension ref="A1:J155"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -724,40 +754,35 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>RENT-MOTORS-08-05-24</t>
+          <t>RENT-MOTORS-06-09-24</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>REX-RENT-08-05-24</t>
+          <t>REX-RENT-06-09-24</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>A-ARENDA-08-05-24</t>
+          <t>A-ARENDA-06-09-24</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>ALMAK-08-05-24</t>
+          <t>STORLET-06-09-24</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>STORLET-08-05-24</t>
+          <t>MIN</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>MIN</t>
+          <t>DELTA</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>DELTA</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>DELTA %</t>
         </is>
@@ -786,7 +811,6 @@
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n"/>
@@ -802,14 +826,13 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
+      <c r="H3" t="n">
+        <v>2634</v>
+      </c>
       <c r="I3" t="n">
-        <v>2634</v>
+        <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K3" t="n">
         <v>0</v>
       </c>
     </row>
@@ -827,14 +850,13 @@
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
+      <c r="H4" t="n">
+        <v>2503</v>
+      </c>
       <c r="I4" t="n">
-        <v>2503</v>
+        <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -852,14 +874,13 @@
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
+      <c r="H5" t="n">
+        <v>2371</v>
+      </c>
       <c r="I5" t="n">
-        <v>2371</v>
+        <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -877,14 +898,13 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
+      <c r="H6" t="n">
+        <v>2187</v>
+      </c>
       <c r="I6" t="n">
-        <v>2187</v>
+        <v>0</v>
       </c>
       <c r="J6" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -902,14 +922,13 @@
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
+      <c r="H7" t="n">
+        <v>2055</v>
+      </c>
       <c r="I7" t="n">
-        <v>2055</v>
+        <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>0</v>
-      </c>
-      <c r="K7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -927,14 +946,13 @@
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
+      <c r="H8" t="n">
+        <v>1976</v>
+      </c>
       <c r="I8" t="n">
-        <v>1976</v>
+        <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>0</v>
-      </c>
-      <c r="K8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -957,7 +975,6 @@
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n"/>
@@ -973,14 +990,13 @@
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
+      <c r="H10" t="n">
+        <v>3292</v>
+      </c>
       <c r="I10" t="n">
-        <v>3292</v>
+        <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>0</v>
-      </c>
-      <c r="K10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -998,14 +1014,13 @@
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
+      <c r="H11" t="n">
+        <v>3128</v>
+      </c>
       <c r="I11" t="n">
-        <v>3128</v>
+        <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>0</v>
-      </c>
-      <c r="K11" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1023,14 +1038,13 @@
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
+      <c r="H12" t="n">
+        <v>2963</v>
+      </c>
       <c r="I12" t="n">
-        <v>2963</v>
+        <v>0</v>
       </c>
       <c r="J12" t="n">
-        <v>0</v>
-      </c>
-      <c r="K12" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1048,14 +1062,13 @@
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
+      <c r="H13" t="n">
+        <v>2733</v>
+      </c>
       <c r="I13" t="n">
-        <v>2733</v>
+        <v>0</v>
       </c>
       <c r="J13" t="n">
-        <v>0</v>
-      </c>
-      <c r="K13" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1073,14 +1086,13 @@
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
+      <c r="H14" t="n">
+        <v>2568</v>
+      </c>
       <c r="I14" t="n">
-        <v>2568</v>
+        <v>0</v>
       </c>
       <c r="J14" t="n">
-        <v>0</v>
-      </c>
-      <c r="K14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1098,14 +1110,13 @@
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
+      <c r="H15" t="n">
+        <v>2469</v>
+      </c>
       <c r="I15" t="n">
-        <v>2469</v>
+        <v>0</v>
       </c>
       <c r="J15" t="n">
-        <v>0</v>
-      </c>
-      <c r="K15" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1128,7 +1139,6 @@
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n"/>
@@ -1144,14 +1154,13 @@
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
+      <c r="H17" t="n">
+        <v>0</v>
+      </c>
       <c r="I17" t="n">
         <v>0</v>
       </c>
-      <c r="J17" t="n">
-        <v>0</v>
-      </c>
-      <c r="K17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n"/>
@@ -1167,14 +1176,13 @@
       <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
+      <c r="H18" t="n">
+        <v>0</v>
+      </c>
       <c r="I18" t="n">
         <v>0</v>
       </c>
-      <c r="J18" t="n">
-        <v>0</v>
-      </c>
-      <c r="K18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n"/>
@@ -1190,14 +1198,13 @@
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
+      <c r="H19" t="n">
+        <v>0</v>
+      </c>
       <c r="I19" t="n">
         <v>0</v>
       </c>
-      <c r="J19" t="n">
-        <v>0</v>
-      </c>
-      <c r="K19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n"/>
@@ -1213,14 +1220,13 @@
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
+      <c r="H20" t="n">
+        <v>0</v>
+      </c>
       <c r="I20" t="n">
         <v>0</v>
       </c>
-      <c r="J20" t="n">
-        <v>0</v>
-      </c>
-      <c r="K20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n"/>
@@ -1236,14 +1242,13 @@
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
+      <c r="H21" t="n">
+        <v>0</v>
+      </c>
       <c r="I21" t="n">
         <v>0</v>
       </c>
-      <c r="J21" t="n">
-        <v>0</v>
-      </c>
-      <c r="K21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n"/>
@@ -1259,14 +1264,13 @@
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
+      <c r="H22" t="n">
+        <v>0</v>
+      </c>
       <c r="I22" t="n">
         <v>0</v>
       </c>
-      <c r="J22" t="n">
-        <v>0</v>
-      </c>
-      <c r="K22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
@@ -1287,15 +1291,10 @@
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>Lada Largus 7 мест MT</t>
-        </is>
-      </c>
+      <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n"/>
@@ -1310,18 +1309,15 @@
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr"/>
-      <c r="G24" t="n">
-        <v>3770</v>
-      </c>
-      <c r="H24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="n">
+        <v>3859</v>
+      </c>
       <c r="I24" t="n">
-        <v>3770</v>
+        <v>0</v>
       </c>
       <c r="J24" t="n">
-        <v>89</v>
-      </c>
-      <c r="K24" t="n">
-        <v>2.31</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
@@ -1337,18 +1333,15 @@
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr"/>
-      <c r="G25" t="n">
-        <v>3570</v>
-      </c>
-      <c r="H25" t="inlineStr"/>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="n">
+        <v>3667</v>
+      </c>
       <c r="I25" t="n">
-        <v>3570</v>
+        <v>0</v>
       </c>
       <c r="J25" t="n">
-        <v>97</v>
-      </c>
-      <c r="K25" t="n">
-        <v>2.65</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
@@ -1364,18 +1357,15 @@
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr"/>
-      <c r="G26" t="n">
-        <v>3270</v>
-      </c>
-      <c r="H26" t="inlineStr"/>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="n">
+        <v>3474</v>
+      </c>
       <c r="I26" t="n">
-        <v>3270</v>
+        <v>0</v>
       </c>
       <c r="J26" t="n">
-        <v>204</v>
-      </c>
-      <c r="K26" t="n">
-        <v>5.87</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
@@ -1391,17 +1381,14 @@
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr"/>
-      <c r="G27" t="n">
-        <v>3270</v>
-      </c>
-      <c r="H27" t="inlineStr"/>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="n">
+        <v>3088</v>
+      </c>
       <c r="I27" t="n">
-        <v>3088</v>
+        <v>0</v>
       </c>
       <c r="J27" t="n">
-        <v>0</v>
-      </c>
-      <c r="K27" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1418,17 +1405,14 @@
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr"/>
-      <c r="G28" t="n">
-        <v>3070</v>
-      </c>
-      <c r="H28" t="inlineStr"/>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="n">
+        <v>2702</v>
+      </c>
       <c r="I28" t="n">
-        <v>2702</v>
+        <v>0</v>
       </c>
       <c r="J28" t="n">
-        <v>0</v>
-      </c>
-      <c r="K28" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1445,17 +1429,14 @@
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr"/>
-      <c r="G29" t="n">
-        <v>3070</v>
-      </c>
-      <c r="H29" t="inlineStr"/>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="n">
+        <v>2702</v>
+      </c>
       <c r="I29" t="n">
-        <v>2702</v>
+        <v>0</v>
       </c>
       <c r="J29" t="n">
-        <v>0</v>
-      </c>
-      <c r="K29" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1482,7 +1463,6 @@
       <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n"/>
@@ -1498,14 +1478,13 @@
       <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr"/>
+      <c r="H31" t="n">
+        <v>2861</v>
+      </c>
       <c r="I31" t="n">
-        <v>2861</v>
+        <v>0</v>
       </c>
       <c r="J31" t="n">
-        <v>0</v>
-      </c>
-      <c r="K31" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1523,14 +1502,13 @@
       <c r="E32" t="inlineStr"/>
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr"/>
+      <c r="H32" t="n">
+        <v>2718</v>
+      </c>
       <c r="I32" t="n">
-        <v>2718</v>
+        <v>0</v>
       </c>
       <c r="J32" t="n">
-        <v>0</v>
-      </c>
-      <c r="K32" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1548,14 +1526,13 @@
       <c r="E33" t="inlineStr"/>
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr"/>
-      <c r="H33" t="inlineStr"/>
+      <c r="H33" t="n">
+        <v>2575</v>
+      </c>
       <c r="I33" t="n">
-        <v>2575</v>
+        <v>0</v>
       </c>
       <c r="J33" t="n">
-        <v>0</v>
-      </c>
-      <c r="K33" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1573,14 +1550,13 @@
       <c r="E34" t="inlineStr"/>
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr"/>
-      <c r="H34" t="inlineStr"/>
+      <c r="H34" t="n">
+        <v>2375</v>
+      </c>
       <c r="I34" t="n">
-        <v>2375</v>
+        <v>0</v>
       </c>
       <c r="J34" t="n">
-        <v>0</v>
-      </c>
-      <c r="K34" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1598,14 +1574,13 @@
       <c r="E35" t="inlineStr"/>
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr"/>
-      <c r="H35" t="inlineStr"/>
+      <c r="H35" t="n">
+        <v>2232</v>
+      </c>
       <c r="I35" t="n">
-        <v>2232</v>
+        <v>0</v>
       </c>
       <c r="J35" t="n">
-        <v>0</v>
-      </c>
-      <c r="K35" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1623,14 +1598,13 @@
       <c r="E36" t="inlineStr"/>
       <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr"/>
-      <c r="H36" t="inlineStr"/>
+      <c r="H36" t="n">
+        <v>2146</v>
+      </c>
       <c r="I36" t="n">
-        <v>2146</v>
+        <v>0</v>
       </c>
       <c r="J36" t="n">
-        <v>0</v>
-      </c>
-      <c r="K36" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1655,11 +1629,7 @@
           <t>Hyundai Solaris</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>Сhangan Alsvin / Renault Logan</t>
-        </is>
-      </c>
+      <c r="E37" t="inlineStr"/>
       <c r="F37" t="inlineStr">
         <is>
           <t>Hyundai  Solaris 1.6  AT</t>
@@ -1667,17 +1637,12 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Hyundai Solaris II Promo</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr">
-        <is>
           <t>Hyundai Solaris sedan</t>
         </is>
       </c>
+      <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr"/>
-      <c r="K37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n"/>
@@ -1690,27 +1655,22 @@
         <v>3576</v>
       </c>
       <c r="D38" t="n">
-        <v>2600</v>
-      </c>
-      <c r="E38" t="n">
-        <v>3800</v>
-      </c>
+        <v>3120</v>
+      </c>
+      <c r="E38" t="inlineStr"/>
       <c r="F38" t="n">
-        <v>3330</v>
+        <v>3430</v>
       </c>
       <c r="G38" t="n">
-        <v>2770</v>
+        <v>2000</v>
       </c>
       <c r="H38" t="n">
         <v>2000</v>
       </c>
       <c r="I38" t="n">
-        <v>2000</v>
+        <v>1576</v>
       </c>
       <c r="J38" t="n">
-        <v>1576</v>
-      </c>
-      <c r="K38" t="n">
         <v>44.07</v>
       </c>
     </row>
@@ -1725,27 +1685,22 @@
         <v>3398</v>
       </c>
       <c r="D39" t="n">
-        <v>2600</v>
-      </c>
-      <c r="E39" t="n">
-        <v>3100</v>
-      </c>
+        <v>3120</v>
+      </c>
+      <c r="E39" t="inlineStr"/>
       <c r="F39" t="n">
-        <v>2990</v>
+        <v>3090</v>
       </c>
       <c r="G39" t="n">
-        <v>2570</v>
+        <v>2000</v>
       </c>
       <c r="H39" t="n">
         <v>2000</v>
       </c>
       <c r="I39" t="n">
-        <v>2000</v>
+        <v>1398</v>
       </c>
       <c r="J39" t="n">
-        <v>1398</v>
-      </c>
-      <c r="K39" t="n">
         <v>41.14</v>
       </c>
     </row>
@@ -1760,27 +1715,22 @@
         <v>3219</v>
       </c>
       <c r="D40" t="n">
-        <v>2500</v>
-      </c>
-      <c r="E40" t="n">
-        <v>2900</v>
-      </c>
+        <v>3000</v>
+      </c>
+      <c r="E40" t="inlineStr"/>
       <c r="F40" t="n">
-        <v>2860</v>
+        <v>2950</v>
       </c>
       <c r="G40" t="n">
-        <v>2470</v>
+        <v>1800</v>
       </c>
       <c r="H40" t="n">
         <v>1800</v>
       </c>
       <c r="I40" t="n">
-        <v>1800</v>
+        <v>1419</v>
       </c>
       <c r="J40" t="n">
-        <v>1419</v>
-      </c>
-      <c r="K40" t="n">
         <v>44.08</v>
       </c>
     </row>
@@ -1795,27 +1745,22 @@
         <v>2969</v>
       </c>
       <c r="D41" t="n">
-        <v>2500</v>
-      </c>
-      <c r="E41" t="n">
-        <v>2600</v>
-      </c>
+        <v>3000</v>
+      </c>
+      <c r="E41" t="inlineStr"/>
       <c r="F41" t="n">
-        <v>2860</v>
+        <v>2950</v>
       </c>
       <c r="G41" t="n">
-        <v>2470</v>
+        <v>1800</v>
       </c>
       <c r="H41" t="n">
         <v>1800</v>
       </c>
       <c r="I41" t="n">
-        <v>1800</v>
+        <v>1169</v>
       </c>
       <c r="J41" t="n">
-        <v>1169</v>
-      </c>
-      <c r="K41" t="n">
         <v>39.37</v>
       </c>
     </row>
@@ -1830,27 +1775,22 @@
         <v>2790</v>
       </c>
       <c r="D42" t="n">
-        <v>2500</v>
-      </c>
-      <c r="E42" t="n">
-        <v>2500</v>
-      </c>
+        <v>3000</v>
+      </c>
+      <c r="E42" t="inlineStr"/>
       <c r="F42" t="n">
-        <v>2660</v>
+        <v>2740</v>
       </c>
       <c r="G42" t="n">
-        <v>2270</v>
+        <v>1500</v>
       </c>
       <c r="H42" t="n">
         <v>1500</v>
       </c>
       <c r="I42" t="n">
-        <v>1500</v>
+        <v>1290</v>
       </c>
       <c r="J42" t="n">
-        <v>1290</v>
-      </c>
-      <c r="K42" t="n">
         <v>46.24</v>
       </c>
     </row>
@@ -1865,27 +1805,22 @@
         <v>2682</v>
       </c>
       <c r="D43" t="n">
-        <v>2200</v>
-      </c>
-      <c r="E43" t="n">
-        <v>2420</v>
-      </c>
+        <v>2640</v>
+      </c>
+      <c r="E43" t="inlineStr"/>
       <c r="F43" t="n">
-        <v>2660</v>
+        <v>2740</v>
       </c>
       <c r="G43" t="n">
-        <v>2270</v>
+        <v>1500</v>
       </c>
       <c r="H43" t="n">
         <v>1500</v>
       </c>
       <c r="I43" t="n">
-        <v>1500</v>
+        <v>1182</v>
       </c>
       <c r="J43" t="n">
-        <v>1182</v>
-      </c>
-      <c r="K43" t="n">
         <v>44.07</v>
       </c>
     </row>
@@ -1912,7 +1847,6 @@
       <c r="H44" t="inlineStr"/>
       <c r="I44" t="inlineStr"/>
       <c r="J44" t="inlineStr"/>
-      <c r="K44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="1" t="n"/>
@@ -1928,14 +1862,13 @@
       <c r="E45" t="inlineStr"/>
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr"/>
-      <c r="H45" t="inlineStr"/>
+      <c r="H45" t="n">
+        <v>3305</v>
+      </c>
       <c r="I45" t="n">
-        <v>3305</v>
+        <v>0</v>
       </c>
       <c r="J45" t="n">
-        <v>0</v>
-      </c>
-      <c r="K45" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1953,14 +1886,13 @@
       <c r="E46" t="inlineStr"/>
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr"/>
-      <c r="H46" t="inlineStr"/>
+      <c r="H46" t="n">
+        <v>3140</v>
+      </c>
       <c r="I46" t="n">
-        <v>3140</v>
+        <v>0</v>
       </c>
       <c r="J46" t="n">
-        <v>0</v>
-      </c>
-      <c r="K46" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1978,14 +1910,13 @@
       <c r="E47" t="inlineStr"/>
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr"/>
-      <c r="H47" t="inlineStr"/>
+      <c r="H47" t="n">
+        <v>2975</v>
+      </c>
       <c r="I47" t="n">
-        <v>2975</v>
+        <v>0</v>
       </c>
       <c r="J47" t="n">
-        <v>0</v>
-      </c>
-      <c r="K47" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2003,14 +1934,13 @@
       <c r="E48" t="inlineStr"/>
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr"/>
-      <c r="H48" t="inlineStr"/>
+      <c r="H48" t="n">
+        <v>2644</v>
+      </c>
       <c r="I48" t="n">
-        <v>2644</v>
+        <v>0</v>
       </c>
       <c r="J48" t="n">
-        <v>0</v>
-      </c>
-      <c r="K48" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2028,14 +1958,13 @@
       <c r="E49" t="inlineStr"/>
       <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr"/>
-      <c r="H49" t="inlineStr"/>
+      <c r="H49" t="n">
+        <v>2314</v>
+      </c>
       <c r="I49" t="n">
-        <v>2314</v>
+        <v>0</v>
       </c>
       <c r="J49" t="n">
-        <v>0</v>
-      </c>
-      <c r="K49" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2053,14 +1982,13 @@
       <c r="E50" t="inlineStr"/>
       <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr"/>
-      <c r="H50" t="inlineStr"/>
+      <c r="H50" t="n">
+        <v>2314</v>
+      </c>
       <c r="I50" t="n">
-        <v>2314</v>
+        <v>0</v>
       </c>
       <c r="J50" t="n">
-        <v>0</v>
-      </c>
-      <c r="K50" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2085,17 +2013,12 @@
       <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Volkswagen Polo АТ Promo</t>
-        </is>
-      </c>
-      <c r="H51" t="inlineStr">
-        <is>
           <t xml:space="preserve">Skoda Rapid </t>
         </is>
       </c>
+      <c r="H51" t="inlineStr"/>
       <c r="I51" t="inlineStr"/>
       <c r="J51" t="inlineStr"/>
-      <c r="K51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="1" t="n"/>
@@ -2111,18 +2034,15 @@
       <c r="E52" t="inlineStr"/>
       <c r="F52" t="inlineStr"/>
       <c r="G52" t="n">
-        <v>2770</v>
+        <v>1800</v>
       </c>
       <c r="H52" t="n">
         <v>1800</v>
       </c>
       <c r="I52" t="n">
-        <v>1800</v>
+        <v>2331</v>
       </c>
       <c r="J52" t="n">
-        <v>2331</v>
-      </c>
-      <c r="K52" t="n">
         <v>56.43</v>
       </c>
     </row>
@@ -2140,18 +2060,15 @@
       <c r="E53" t="inlineStr"/>
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="n">
-        <v>2570</v>
+        <v>1800</v>
       </c>
       <c r="H53" t="n">
         <v>1800</v>
       </c>
       <c r="I53" t="n">
-        <v>1800</v>
+        <v>2125</v>
       </c>
       <c r="J53" t="n">
-        <v>2125</v>
-      </c>
-      <c r="K53" t="n">
         <v>54.14</v>
       </c>
     </row>
@@ -2169,18 +2086,15 @@
       <c r="E54" t="inlineStr"/>
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="n">
-        <v>2470</v>
+        <v>1600</v>
       </c>
       <c r="H54" t="n">
         <v>1600</v>
       </c>
       <c r="I54" t="n">
-        <v>1600</v>
+        <v>2118</v>
       </c>
       <c r="J54" t="n">
-        <v>2118</v>
-      </c>
-      <c r="K54" t="n">
         <v>56.97</v>
       </c>
     </row>
@@ -2198,18 +2112,15 @@
       <c r="E55" t="inlineStr"/>
       <c r="F55" t="inlineStr"/>
       <c r="G55" t="n">
-        <v>2470</v>
+        <v>1600</v>
       </c>
       <c r="H55" t="n">
         <v>1600</v>
       </c>
       <c r="I55" t="n">
-        <v>1600</v>
+        <v>1705</v>
       </c>
       <c r="J55" t="n">
-        <v>1705</v>
-      </c>
-      <c r="K55" t="n">
         <v>51.59</v>
       </c>
     </row>
@@ -2227,18 +2138,15 @@
       <c r="E56" t="inlineStr"/>
       <c r="F56" t="inlineStr"/>
       <c r="G56" t="n">
-        <v>2270</v>
+        <v>1400</v>
       </c>
       <c r="H56" t="n">
         <v>1400</v>
       </c>
       <c r="I56" t="n">
-        <v>1400</v>
+        <v>1492</v>
       </c>
       <c r="J56" t="n">
-        <v>1492</v>
-      </c>
-      <c r="K56" t="n">
         <v>51.59</v>
       </c>
     </row>
@@ -2256,18 +2164,15 @@
       <c r="E57" t="inlineStr"/>
       <c r="F57" t="inlineStr"/>
       <c r="G57" t="n">
-        <v>2270</v>
+        <v>1400</v>
       </c>
       <c r="H57" t="n">
         <v>1400</v>
       </c>
       <c r="I57" t="n">
-        <v>1400</v>
+        <v>1492</v>
       </c>
       <c r="J57" t="n">
-        <v>1492</v>
-      </c>
-      <c r="K57" t="n">
         <v>51.59</v>
       </c>
     </row>
@@ -2294,15 +2199,14 @@
       </c>
       <c r="E58" t="inlineStr"/>
       <c r="F58" t="inlineStr"/>
-      <c r="G58" t="inlineStr"/>
-      <c r="H58" t="inlineStr">
+      <c r="G58" t="inlineStr">
         <is>
           <t>Skoda Octavia</t>
         </is>
       </c>
+      <c r="H58" t="inlineStr"/>
       <c r="I58" t="inlineStr"/>
       <c r="J58" t="inlineStr"/>
-      <c r="K58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="1" t="n"/>
@@ -2315,22 +2219,21 @@
         <v>3690</v>
       </c>
       <c r="D59" t="n">
-        <v>3000</v>
+        <v>3600</v>
       </c>
       <c r="E59" t="inlineStr"/>
       <c r="F59" t="inlineStr"/>
-      <c r="G59" t="inlineStr"/>
+      <c r="G59" t="n">
+        <v>3200</v>
+      </c>
       <c r="H59" t="n">
         <v>3200</v>
       </c>
       <c r="I59" t="n">
-        <v>3000</v>
+        <v>490</v>
       </c>
       <c r="J59" t="n">
-        <v>690</v>
-      </c>
-      <c r="K59" t="n">
-        <v>18.7</v>
+        <v>13.28</v>
       </c>
     </row>
     <row r="60">
@@ -2344,22 +2247,21 @@
         <v>3506</v>
       </c>
       <c r="D60" t="n">
-        <v>3000</v>
+        <v>3600</v>
       </c>
       <c r="E60" t="inlineStr"/>
       <c r="F60" t="inlineStr"/>
-      <c r="G60" t="inlineStr"/>
+      <c r="G60" t="n">
+        <v>3200</v>
+      </c>
       <c r="H60" t="n">
         <v>3200</v>
       </c>
       <c r="I60" t="n">
-        <v>3000</v>
+        <v>306</v>
       </c>
       <c r="J60" t="n">
-        <v>506</v>
-      </c>
-      <c r="K60" t="n">
-        <v>14.43</v>
+        <v>8.73</v>
       </c>
     </row>
     <row r="61">
@@ -2373,22 +2275,21 @@
         <v>3321</v>
       </c>
       <c r="D61" t="n">
-        <v>2600</v>
+        <v>3120</v>
       </c>
       <c r="E61" t="inlineStr"/>
       <c r="F61" t="inlineStr"/>
-      <c r="G61" t="inlineStr"/>
+      <c r="G61" t="n">
+        <v>2900</v>
+      </c>
       <c r="H61" t="n">
         <v>2900</v>
       </c>
       <c r="I61" t="n">
-        <v>2600</v>
+        <v>421</v>
       </c>
       <c r="J61" t="n">
-        <v>721</v>
-      </c>
-      <c r="K61" t="n">
-        <v>21.71</v>
+        <v>12.68</v>
       </c>
     </row>
     <row r="62">
@@ -2402,22 +2303,21 @@
         <v>2952</v>
       </c>
       <c r="D62" t="n">
-        <v>2600</v>
+        <v>3120</v>
       </c>
       <c r="E62" t="inlineStr"/>
       <c r="F62" t="inlineStr"/>
-      <c r="G62" t="inlineStr"/>
+      <c r="G62" t="n">
+        <v>2900</v>
+      </c>
       <c r="H62" t="n">
         <v>2900</v>
       </c>
       <c r="I62" t="n">
-        <v>2600</v>
+        <v>52</v>
       </c>
       <c r="J62" t="n">
-        <v>352</v>
-      </c>
-      <c r="K62" t="n">
-        <v>11.92</v>
+        <v>1.76</v>
       </c>
     </row>
     <row r="63">
@@ -2431,21 +2331,20 @@
         <v>2583</v>
       </c>
       <c r="D63" t="n">
-        <v>2600</v>
+        <v>3120</v>
       </c>
       <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr"/>
-      <c r="G63" t="inlineStr"/>
+      <c r="G63" t="n">
+        <v>2500</v>
+      </c>
       <c r="H63" t="n">
         <v>2500</v>
       </c>
       <c r="I63" t="n">
-        <v>2500</v>
+        <v>83</v>
       </c>
       <c r="J63" t="n">
-        <v>83</v>
-      </c>
-      <c r="K63" t="n">
         <v>3.21</v>
       </c>
     </row>
@@ -2460,22 +2359,21 @@
         <v>2583</v>
       </c>
       <c r="D64" t="n">
-        <v>2400</v>
+        <v>2880</v>
       </c>
       <c r="E64" t="inlineStr"/>
       <c r="F64" t="inlineStr"/>
-      <c r="G64" t="inlineStr"/>
+      <c r="G64" t="n">
+        <v>2500</v>
+      </c>
       <c r="H64" t="n">
         <v>2500</v>
       </c>
       <c r="I64" t="n">
-        <v>2400</v>
+        <v>83</v>
       </c>
       <c r="J64" t="n">
-        <v>183</v>
-      </c>
-      <c r="K64" t="n">
-        <v>7.08</v>
+        <v>3.21</v>
       </c>
     </row>
     <row r="65">
@@ -2495,17 +2393,20 @@
         </is>
       </c>
       <c r="D65" t="inlineStr"/>
-      <c r="E65" t="inlineStr"/>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Changan UNI-V</t>
+        </is>
+      </c>
       <c r="F65" t="inlineStr"/>
-      <c r="G65" t="inlineStr"/>
-      <c r="H65" t="inlineStr">
+      <c r="G65" t="inlineStr">
         <is>
           <t>Kia Ceed</t>
         </is>
       </c>
+      <c r="H65" t="inlineStr"/>
       <c r="I65" t="inlineStr"/>
       <c r="J65" t="inlineStr"/>
-      <c r="K65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="1" t="n"/>
@@ -2518,19 +2419,20 @@
         <v>4341</v>
       </c>
       <c r="D66" t="inlineStr"/>
-      <c r="E66" t="inlineStr"/>
+      <c r="E66" t="n">
+        <v>8273</v>
+      </c>
       <c r="F66" t="inlineStr"/>
-      <c r="G66" t="inlineStr"/>
+      <c r="G66" t="n">
+        <v>2200</v>
+      </c>
       <c r="H66" t="n">
         <v>2200</v>
       </c>
       <c r="I66" t="n">
-        <v>2200</v>
+        <v>2141</v>
       </c>
       <c r="J66" t="n">
-        <v>2141</v>
-      </c>
-      <c r="K66" t="n">
         <v>49.32</v>
       </c>
     </row>
@@ -2545,19 +2447,20 @@
         <v>4124</v>
       </c>
       <c r="D67" t="inlineStr"/>
-      <c r="E67" t="inlineStr"/>
+      <c r="E67" t="n">
+        <v>6702</v>
+      </c>
       <c r="F67" t="inlineStr"/>
-      <c r="G67" t="inlineStr"/>
+      <c r="G67" t="n">
+        <v>2200</v>
+      </c>
       <c r="H67" t="n">
         <v>2200</v>
       </c>
       <c r="I67" t="n">
-        <v>2200</v>
+        <v>1924</v>
       </c>
       <c r="J67" t="n">
-        <v>1924</v>
-      </c>
-      <c r="K67" t="n">
         <v>46.65</v>
       </c>
     </row>
@@ -2572,19 +2475,20 @@
         <v>3907</v>
       </c>
       <c r="D68" t="inlineStr"/>
-      <c r="E68" t="inlineStr"/>
+      <c r="E68" t="n">
+        <v>5969</v>
+      </c>
       <c r="F68" t="inlineStr"/>
-      <c r="G68" t="inlineStr"/>
+      <c r="G68" t="n">
+        <v>2100</v>
+      </c>
       <c r="H68" t="n">
         <v>2100</v>
       </c>
       <c r="I68" t="n">
-        <v>2100</v>
+        <v>1807</v>
       </c>
       <c r="J68" t="n">
-        <v>1807</v>
-      </c>
-      <c r="K68" t="n">
         <v>46.25</v>
       </c>
     </row>
@@ -2599,19 +2503,20 @@
         <v>3473</v>
       </c>
       <c r="D69" t="inlineStr"/>
-      <c r="E69" t="inlineStr"/>
+      <c r="E69" t="n">
+        <v>5026.57</v>
+      </c>
       <c r="F69" t="inlineStr"/>
-      <c r="G69" t="inlineStr"/>
+      <c r="G69" t="n">
+        <v>2100</v>
+      </c>
       <c r="H69" t="n">
         <v>2100</v>
       </c>
       <c r="I69" t="n">
-        <v>2100</v>
+        <v>1373</v>
       </c>
       <c r="J69" t="n">
-        <v>1373</v>
-      </c>
-      <c r="K69" t="n">
         <v>39.53</v>
       </c>
     </row>
@@ -2626,19 +2531,20 @@
         <v>3039</v>
       </c>
       <c r="D70" t="inlineStr"/>
-      <c r="E70" t="inlineStr"/>
+      <c r="E70" t="n">
+        <v>4817.14</v>
+      </c>
       <c r="F70" t="inlineStr"/>
-      <c r="G70" t="inlineStr"/>
+      <c r="G70" t="n">
+        <v>2000</v>
+      </c>
       <c r="H70" t="n">
         <v>2000</v>
       </c>
       <c r="I70" t="n">
-        <v>2000</v>
+        <v>1039</v>
       </c>
       <c r="J70" t="n">
-        <v>1039</v>
-      </c>
-      <c r="K70" t="n">
         <v>34.19</v>
       </c>
     </row>
@@ -2653,19 +2559,20 @@
         <v>3039</v>
       </c>
       <c r="D71" t="inlineStr"/>
-      <c r="E71" t="inlineStr"/>
+      <c r="E71" t="n">
+        <v>4293.53</v>
+      </c>
       <c r="F71" t="inlineStr"/>
-      <c r="G71" t="inlineStr"/>
+      <c r="G71" t="n">
+        <v>2000</v>
+      </c>
       <c r="H71" t="n">
         <v>2000</v>
       </c>
       <c r="I71" t="n">
-        <v>2000</v>
+        <v>1039</v>
       </c>
       <c r="J71" t="n">
-        <v>1039</v>
-      </c>
-      <c r="K71" t="n">
         <v>34.19</v>
       </c>
     </row>
@@ -2697,22 +2604,17 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>Hyundai Sonata VIII 2.5</t>
+          <t>Kia K5</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Hyundai Sonata AT Promo</t>
-        </is>
-      </c>
-      <c r="H72" t="inlineStr">
-        <is>
           <t>Hyundai i40</t>
         </is>
       </c>
+      <c r="H72" t="inlineStr"/>
       <c r="I72" t="inlineStr"/>
       <c r="J72" t="inlineStr"/>
-      <c r="K72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="1" t="n"/>
@@ -2725,27 +2627,24 @@
         <v>5001</v>
       </c>
       <c r="D73" t="n">
-        <v>4300</v>
+        <v>5160</v>
       </c>
       <c r="E73" t="n">
-        <v>9100</v>
+        <v>9530</v>
       </c>
       <c r="F73" t="n">
-        <v>3900</v>
+        <v>5000</v>
       </c>
       <c r="G73" t="n">
-        <v>4370</v>
+        <v>2500</v>
       </c>
       <c r="H73" t="n">
         <v>2500</v>
       </c>
       <c r="I73" t="n">
-        <v>2500</v>
+        <v>2501</v>
       </c>
       <c r="J73" t="n">
-        <v>2501</v>
-      </c>
-      <c r="K73" t="n">
         <v>50.01</v>
       </c>
     </row>
@@ -2760,27 +2659,24 @@
         <v>4751</v>
       </c>
       <c r="D74" t="n">
-        <v>4300</v>
+        <v>5160</v>
       </c>
       <c r="E74" t="n">
-        <v>8100</v>
+        <v>8482.33</v>
       </c>
       <c r="F74" t="n">
-        <v>3710</v>
+        <v>4750</v>
       </c>
       <c r="G74" t="n">
-        <v>4070</v>
+        <v>2500</v>
       </c>
       <c r="H74" t="n">
         <v>2500</v>
       </c>
       <c r="I74" t="n">
-        <v>2500</v>
+        <v>2251</v>
       </c>
       <c r="J74" t="n">
-        <v>2251</v>
-      </c>
-      <c r="K74" t="n">
         <v>47.38</v>
       </c>
     </row>
@@ -2795,27 +2691,24 @@
         <v>4501</v>
       </c>
       <c r="D75" t="n">
-        <v>3700</v>
+        <v>4440</v>
       </c>
       <c r="E75" t="n">
-        <v>6250</v>
+        <v>6545</v>
       </c>
       <c r="F75" t="n">
-        <v>3510</v>
+        <v>4500</v>
       </c>
       <c r="G75" t="n">
-        <v>3670</v>
+        <v>2400</v>
       </c>
       <c r="H75" t="n">
         <v>2400</v>
       </c>
       <c r="I75" t="n">
-        <v>2400</v>
+        <v>2101</v>
       </c>
       <c r="J75" t="n">
-        <v>2101</v>
-      </c>
-      <c r="K75" t="n">
         <v>46.68</v>
       </c>
     </row>
@@ -2830,27 +2723,24 @@
         <v>4001</v>
       </c>
       <c r="D76" t="n">
-        <v>3700</v>
+        <v>4440</v>
       </c>
       <c r="E76" t="n">
-        <v>5500</v>
+        <v>5759.57</v>
       </c>
       <c r="F76" t="n">
-        <v>3510</v>
+        <v>4500</v>
       </c>
       <c r="G76" t="n">
-        <v>3670</v>
+        <v>2400</v>
       </c>
       <c r="H76" t="n">
         <v>2400</v>
       </c>
       <c r="I76" t="n">
-        <v>2400</v>
+        <v>1601</v>
       </c>
       <c r="J76" t="n">
-        <v>1601</v>
-      </c>
-      <c r="K76" t="n">
         <v>40.01</v>
       </c>
     </row>
@@ -2865,27 +2755,24 @@
         <v>3501</v>
       </c>
       <c r="D77" t="n">
-        <v>3700</v>
+        <v>4440</v>
       </c>
       <c r="E77" t="n">
-        <v>5300</v>
+        <v>5550.14</v>
       </c>
       <c r="F77" t="n">
-        <v>3347.62</v>
+        <v>4250</v>
       </c>
       <c r="G77" t="n">
-        <v>3570</v>
+        <v>1900</v>
       </c>
       <c r="H77" t="n">
         <v>1900</v>
       </c>
       <c r="I77" t="n">
-        <v>1900</v>
+        <v>1601</v>
       </c>
       <c r="J77" t="n">
-        <v>1601</v>
-      </c>
-      <c r="K77" t="n">
         <v>45.73</v>
       </c>
     </row>
@@ -2900,27 +2787,24 @@
         <v>3501</v>
       </c>
       <c r="D78" t="n">
-        <v>3300</v>
+        <v>3960</v>
       </c>
       <c r="E78" t="n">
-        <v>4800</v>
+        <v>5026.57</v>
       </c>
       <c r="F78" t="n">
-        <v>3426.33</v>
+        <v>4250</v>
       </c>
       <c r="G78" t="n">
-        <v>3570</v>
+        <v>1900</v>
       </c>
       <c r="H78" t="n">
         <v>1900</v>
       </c>
       <c r="I78" t="n">
-        <v>1900</v>
+        <v>1601</v>
       </c>
       <c r="J78" t="n">
-        <v>1601</v>
-      </c>
-      <c r="K78" t="n">
         <v>45.73</v>
       </c>
     </row>
@@ -2943,7 +2827,6 @@
       <c r="H79" t="inlineStr"/>
       <c r="I79" t="inlineStr"/>
       <c r="J79" t="inlineStr"/>
-      <c r="K79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="1" t="n"/>
@@ -2959,14 +2842,13 @@
       <c r="E80" t="inlineStr"/>
       <c r="F80" t="inlineStr"/>
       <c r="G80" t="inlineStr"/>
-      <c r="H80" t="inlineStr"/>
+      <c r="H80" t="n">
+        <v>5556</v>
+      </c>
       <c r="I80" t="n">
-        <v>5556</v>
+        <v>0</v>
       </c>
       <c r="J80" t="n">
-        <v>0</v>
-      </c>
-      <c r="K80" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2984,14 +2866,13 @@
       <c r="E81" t="inlineStr"/>
       <c r="F81" t="inlineStr"/>
       <c r="G81" t="inlineStr"/>
-      <c r="H81" t="inlineStr"/>
+      <c r="H81" t="n">
+        <v>5279</v>
+      </c>
       <c r="I81" t="n">
-        <v>5279</v>
+        <v>0</v>
       </c>
       <c r="J81" t="n">
-        <v>0</v>
-      </c>
-      <c r="K81" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3009,14 +2890,13 @@
       <c r="E82" t="inlineStr"/>
       <c r="F82" t="inlineStr"/>
       <c r="G82" t="inlineStr"/>
-      <c r="H82" t="inlineStr"/>
+      <c r="H82" t="n">
+        <v>5001</v>
+      </c>
       <c r="I82" t="n">
-        <v>5001</v>
+        <v>0</v>
       </c>
       <c r="J82" t="n">
-        <v>0</v>
-      </c>
-      <c r="K82" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3034,14 +2914,13 @@
       <c r="E83" t="inlineStr"/>
       <c r="F83" t="inlineStr"/>
       <c r="G83" t="inlineStr"/>
-      <c r="H83" t="inlineStr"/>
+      <c r="H83" t="n">
+        <v>4445</v>
+      </c>
       <c r="I83" t="n">
-        <v>4445</v>
+        <v>0</v>
       </c>
       <c r="J83" t="n">
-        <v>0</v>
-      </c>
-      <c r="K83" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3059,14 +2938,13 @@
       <c r="E84" t="inlineStr"/>
       <c r="F84" t="inlineStr"/>
       <c r="G84" t="inlineStr"/>
-      <c r="H84" t="inlineStr"/>
+      <c r="H84" t="n">
+        <v>3890</v>
+      </c>
       <c r="I84" t="n">
-        <v>3890</v>
+        <v>0</v>
       </c>
       <c r="J84" t="n">
-        <v>0</v>
-      </c>
-      <c r="K84" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3084,14 +2962,13 @@
       <c r="E85" t="inlineStr"/>
       <c r="F85" t="inlineStr"/>
       <c r="G85" t="inlineStr"/>
-      <c r="H85" t="inlineStr"/>
+      <c r="H85" t="n">
+        <v>3890</v>
+      </c>
       <c r="I85" t="n">
-        <v>3890</v>
+        <v>0</v>
       </c>
       <c r="J85" t="n">
-        <v>0</v>
-      </c>
-      <c r="K85" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3116,17 +2993,12 @@
       <c r="F86" t="inlineStr"/>
       <c r="G86" t="inlineStr">
         <is>
-          <t>Hyundai Creta AT</t>
-        </is>
-      </c>
-      <c r="H86" t="inlineStr">
-        <is>
           <t>Renault Kaptur</t>
         </is>
       </c>
+      <c r="H86" t="inlineStr"/>
       <c r="I86" t="inlineStr"/>
       <c r="J86" t="inlineStr"/>
-      <c r="K86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="1" t="n"/>
@@ -3142,18 +3014,15 @@
       <c r="E87" t="inlineStr"/>
       <c r="F87" t="inlineStr"/>
       <c r="G87" t="n">
-        <v>3970</v>
+        <v>2200</v>
       </c>
       <c r="H87" t="n">
         <v>2200</v>
       </c>
       <c r="I87" t="n">
-        <v>2200</v>
+        <v>1839</v>
       </c>
       <c r="J87" t="n">
-        <v>1839</v>
-      </c>
-      <c r="K87" t="n">
         <v>45.53</v>
       </c>
     </row>
@@ -3171,18 +3040,15 @@
       <c r="E88" t="inlineStr"/>
       <c r="F88" t="inlineStr"/>
       <c r="G88" t="n">
-        <v>3770</v>
+        <v>2200</v>
       </c>
       <c r="H88" t="n">
         <v>2200</v>
       </c>
       <c r="I88" t="n">
-        <v>2200</v>
+        <v>1638</v>
       </c>
       <c r="J88" t="n">
-        <v>1638</v>
-      </c>
-      <c r="K88" t="n">
         <v>42.68</v>
       </c>
     </row>
@@ -3200,18 +3066,15 @@
       <c r="E89" t="inlineStr"/>
       <c r="F89" t="inlineStr"/>
       <c r="G89" t="n">
-        <v>3470</v>
+        <v>1900</v>
       </c>
       <c r="H89" t="n">
         <v>1900</v>
       </c>
       <c r="I89" t="n">
-        <v>1900</v>
+        <v>1736</v>
       </c>
       <c r="J89" t="n">
-        <v>1736</v>
-      </c>
-      <c r="K89" t="n">
         <v>47.74</v>
       </c>
     </row>
@@ -3229,18 +3092,15 @@
       <c r="E90" t="inlineStr"/>
       <c r="F90" t="inlineStr"/>
       <c r="G90" t="n">
-        <v>3470</v>
+        <v>1900</v>
       </c>
       <c r="H90" t="n">
         <v>1900</v>
       </c>
       <c r="I90" t="n">
-        <v>1900</v>
+        <v>1332</v>
       </c>
       <c r="J90" t="n">
-        <v>1332</v>
-      </c>
-      <c r="K90" t="n">
         <v>41.21</v>
       </c>
     </row>
@@ -3258,18 +3118,15 @@
       <c r="E91" t="inlineStr"/>
       <c r="F91" t="inlineStr"/>
       <c r="G91" t="n">
-        <v>3270</v>
+        <v>1600</v>
       </c>
       <c r="H91" t="n">
         <v>1600</v>
       </c>
       <c r="I91" t="n">
-        <v>1600</v>
+        <v>1430</v>
       </c>
       <c r="J91" t="n">
-        <v>1430</v>
-      </c>
-      <c r="K91" t="n">
         <v>47.19</v>
       </c>
     </row>
@@ -3287,18 +3144,15 @@
       <c r="E92" t="inlineStr"/>
       <c r="F92" t="inlineStr"/>
       <c r="G92" t="n">
-        <v>3270</v>
+        <v>1600</v>
       </c>
       <c r="H92" t="n">
         <v>1600</v>
       </c>
       <c r="I92" t="n">
-        <v>1600</v>
+        <v>1228</v>
       </c>
       <c r="J92" t="n">
-        <v>1228</v>
-      </c>
-      <c r="K92" t="n">
         <v>43.42</v>
       </c>
     </row>
@@ -3319,21 +3173,12 @@
         </is>
       </c>
       <c r="D93" t="inlineStr"/>
-      <c r="E93" t="inlineStr">
-        <is>
-          <t>Сhery Tiggo 4</t>
-        </is>
-      </c>
+      <c r="E93" t="inlineStr"/>
       <c r="F93" t="inlineStr"/>
-      <c r="G93" t="inlineStr">
-        <is>
-          <t>Renault Duster 4WD AT</t>
-        </is>
-      </c>
+      <c r="G93" t="inlineStr"/>
       <c r="H93" t="inlineStr"/>
       <c r="I93" t="inlineStr"/>
       <c r="J93" t="inlineStr"/>
-      <c r="K93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="1" t="n"/>
@@ -3346,22 +3191,17 @@
         <v>4487</v>
       </c>
       <c r="D94" t="inlineStr"/>
-      <c r="E94" t="n">
-        <v>5500</v>
-      </c>
+      <c r="E94" t="inlineStr"/>
       <c r="F94" t="inlineStr"/>
-      <c r="G94" t="n">
-        <v>3970</v>
-      </c>
-      <c r="H94" t="inlineStr"/>
+      <c r="G94" t="inlineStr"/>
+      <c r="H94" t="n">
+        <v>4487</v>
+      </c>
       <c r="I94" t="n">
-        <v>3970</v>
+        <v>0</v>
       </c>
       <c r="J94" t="n">
-        <v>517</v>
-      </c>
-      <c r="K94" t="n">
-        <v>11.52</v>
+        <v>0</v>
       </c>
     </row>
     <row r="95">
@@ -3375,22 +3215,17 @@
         <v>4263</v>
       </c>
       <c r="D95" t="inlineStr"/>
-      <c r="E95" t="n">
-        <v>4100</v>
-      </c>
+      <c r="E95" t="inlineStr"/>
       <c r="F95" t="inlineStr"/>
-      <c r="G95" t="n">
-        <v>3770</v>
-      </c>
-      <c r="H95" t="inlineStr"/>
+      <c r="G95" t="inlineStr"/>
+      <c r="H95" t="n">
+        <v>4263</v>
+      </c>
       <c r="I95" t="n">
-        <v>3770</v>
+        <v>0</v>
       </c>
       <c r="J95" t="n">
-        <v>493</v>
-      </c>
-      <c r="K95" t="n">
-        <v>11.56</v>
+        <v>0</v>
       </c>
     </row>
     <row r="96">
@@ -3404,22 +3239,17 @@
         <v>4039</v>
       </c>
       <c r="D96" t="inlineStr"/>
-      <c r="E96" t="n">
-        <v>3800</v>
-      </c>
+      <c r="E96" t="inlineStr"/>
       <c r="F96" t="inlineStr"/>
-      <c r="G96" t="n">
-        <v>3470</v>
-      </c>
-      <c r="H96" t="inlineStr"/>
+      <c r="G96" t="inlineStr"/>
+      <c r="H96" t="n">
+        <v>4039</v>
+      </c>
       <c r="I96" t="n">
-        <v>3470</v>
+        <v>0</v>
       </c>
       <c r="J96" t="n">
-        <v>569</v>
-      </c>
-      <c r="K96" t="n">
-        <v>14.09</v>
+        <v>0</v>
       </c>
     </row>
     <row r="97">
@@ -3433,22 +3263,17 @@
         <v>3590</v>
       </c>
       <c r="D97" t="inlineStr"/>
-      <c r="E97" t="n">
-        <v>3300</v>
-      </c>
+      <c r="E97" t="inlineStr"/>
       <c r="F97" t="inlineStr"/>
-      <c r="G97" t="n">
-        <v>3470</v>
-      </c>
-      <c r="H97" t="inlineStr"/>
+      <c r="G97" t="inlineStr"/>
+      <c r="H97" t="n">
+        <v>3590</v>
+      </c>
       <c r="I97" t="n">
-        <v>3300</v>
+        <v>0</v>
       </c>
       <c r="J97" t="n">
-        <v>290</v>
-      </c>
-      <c r="K97" t="n">
-        <v>8.08</v>
+        <v>0</v>
       </c>
     </row>
     <row r="98">
@@ -3462,22 +3287,17 @@
         <v>3366</v>
       </c>
       <c r="D98" t="inlineStr"/>
-      <c r="E98" t="n">
-        <v>3100</v>
-      </c>
+      <c r="E98" t="inlineStr"/>
       <c r="F98" t="inlineStr"/>
-      <c r="G98" t="n">
-        <v>3270</v>
-      </c>
-      <c r="H98" t="inlineStr"/>
+      <c r="G98" t="inlineStr"/>
+      <c r="H98" t="n">
+        <v>3366</v>
+      </c>
       <c r="I98" t="n">
-        <v>3100</v>
+        <v>0</v>
       </c>
       <c r="J98" t="n">
-        <v>266</v>
-      </c>
-      <c r="K98" t="n">
-        <v>7.9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="99">
@@ -3491,22 +3311,17 @@
         <v>3141</v>
       </c>
       <c r="D99" t="inlineStr"/>
-      <c r="E99" t="n">
-        <v>2800</v>
-      </c>
+      <c r="E99" t="inlineStr"/>
       <c r="F99" t="inlineStr"/>
-      <c r="G99" t="n">
-        <v>3270</v>
-      </c>
-      <c r="H99" t="inlineStr"/>
+      <c r="G99" t="inlineStr"/>
+      <c r="H99" t="n">
+        <v>3141</v>
+      </c>
       <c r="I99" t="n">
-        <v>2800</v>
+        <v>0</v>
       </c>
       <c r="J99" t="n">
-        <v>341</v>
-      </c>
-      <c r="K99" t="n">
-        <v>10.86</v>
+        <v>0</v>
       </c>
     </row>
     <row r="100">
@@ -3528,7 +3343,6 @@
       <c r="H100" t="inlineStr"/>
       <c r="I100" t="inlineStr"/>
       <c r="J100" t="inlineStr"/>
-      <c r="K100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="1" t="n"/>
@@ -3544,14 +3358,13 @@
       <c r="E101" t="inlineStr"/>
       <c r="F101" t="inlineStr"/>
       <c r="G101" t="inlineStr"/>
-      <c r="H101" t="inlineStr"/>
+      <c r="H101" t="n">
+        <v>0</v>
+      </c>
       <c r="I101" t="n">
         <v>0</v>
       </c>
-      <c r="J101" t="n">
-        <v>0</v>
-      </c>
-      <c r="K101" t="inlineStr"/>
+      <c r="J101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" s="1" t="n"/>
@@ -3567,14 +3380,13 @@
       <c r="E102" t="inlineStr"/>
       <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr"/>
-      <c r="H102" t="inlineStr"/>
+      <c r="H102" t="n">
+        <v>0</v>
+      </c>
       <c r="I102" t="n">
         <v>0</v>
       </c>
-      <c r="J102" t="n">
-        <v>0</v>
-      </c>
-      <c r="K102" t="inlineStr"/>
+      <c r="J102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" s="1" t="n"/>
@@ -3590,14 +3402,13 @@
       <c r="E103" t="inlineStr"/>
       <c r="F103" t="inlineStr"/>
       <c r="G103" t="inlineStr"/>
-      <c r="H103" t="inlineStr"/>
+      <c r="H103" t="n">
+        <v>0</v>
+      </c>
       <c r="I103" t="n">
         <v>0</v>
       </c>
-      <c r="J103" t="n">
-        <v>0</v>
-      </c>
-      <c r="K103" t="inlineStr"/>
+      <c r="J103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" s="1" t="n"/>
@@ -3613,14 +3424,13 @@
       <c r="E104" t="inlineStr"/>
       <c r="F104" t="inlineStr"/>
       <c r="G104" t="inlineStr"/>
-      <c r="H104" t="inlineStr"/>
+      <c r="H104" t="n">
+        <v>0</v>
+      </c>
       <c r="I104" t="n">
         <v>0</v>
       </c>
-      <c r="J104" t="n">
-        <v>0</v>
-      </c>
-      <c r="K104" t="inlineStr"/>
+      <c r="J104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" s="1" t="n"/>
@@ -3636,14 +3446,13 @@
       <c r="E105" t="inlineStr"/>
       <c r="F105" t="inlineStr"/>
       <c r="G105" t="inlineStr"/>
-      <c r="H105" t="inlineStr"/>
+      <c r="H105" t="n">
+        <v>0</v>
+      </c>
       <c r="I105" t="n">
         <v>0</v>
       </c>
-      <c r="J105" t="n">
-        <v>0</v>
-      </c>
-      <c r="K105" t="inlineStr"/>
+      <c r="J105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" s="1" t="n"/>
@@ -3659,14 +3468,13 @@
       <c r="E106" t="inlineStr"/>
       <c r="F106" t="inlineStr"/>
       <c r="G106" t="inlineStr"/>
-      <c r="H106" t="inlineStr"/>
+      <c r="H106" t="n">
+        <v>0</v>
+      </c>
       <c r="I106" t="n">
         <v>0</v>
       </c>
-      <c r="J106" t="n">
-        <v>0</v>
-      </c>
-      <c r="K106" t="inlineStr"/>
+      <c r="J106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" s="1" t="inlineStr">
@@ -3698,17 +3506,12 @@
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>Hyundai Creta II AT Promo</t>
-        </is>
-      </c>
-      <c r="H107" t="inlineStr">
-        <is>
           <t>Toyota CH R</t>
         </is>
       </c>
+      <c r="H107" t="inlineStr"/>
       <c r="I107" t="inlineStr"/>
       <c r="J107" t="inlineStr"/>
-      <c r="K107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" s="1" t="n"/>
@@ -3721,26 +3524,23 @@
         <v>4701</v>
       </c>
       <c r="D108" t="n">
-        <v>3700</v>
+        <v>4440</v>
       </c>
       <c r="E108" t="inlineStr"/>
       <c r="F108" t="n">
         <v>3900</v>
       </c>
       <c r="G108" t="n">
-        <v>4170</v>
+        <v>3900</v>
       </c>
       <c r="H108" t="n">
         <v>3900</v>
       </c>
       <c r="I108" t="n">
-        <v>3700</v>
+        <v>801</v>
       </c>
       <c r="J108" t="n">
-        <v>1001</v>
-      </c>
-      <c r="K108" t="n">
-        <v>21.29</v>
+        <v>17.04</v>
       </c>
     </row>
     <row r="109">
@@ -3754,25 +3554,22 @@
         <v>4466</v>
       </c>
       <c r="D109" t="n">
-        <v>3700</v>
+        <v>4440</v>
       </c>
       <c r="E109" t="inlineStr"/>
       <c r="F109" t="n">
         <v>3700</v>
       </c>
       <c r="G109" t="n">
-        <v>3870</v>
+        <v>3900</v>
       </c>
       <c r="H109" t="n">
-        <v>3900</v>
+        <v>3700</v>
       </c>
       <c r="I109" t="n">
-        <v>3700</v>
+        <v>766</v>
       </c>
       <c r="J109" t="n">
-        <v>766</v>
-      </c>
-      <c r="K109" t="n">
         <v>17.15</v>
       </c>
     </row>
@@ -3787,26 +3584,23 @@
         <v>4231</v>
       </c>
       <c r="D110" t="n">
-        <v>3300</v>
+        <v>3960</v>
       </c>
       <c r="E110" t="inlineStr"/>
       <c r="F110" t="n">
         <v>3510</v>
       </c>
       <c r="G110" t="n">
-        <v>3570</v>
+        <v>3500</v>
       </c>
       <c r="H110" t="n">
         <v>3500</v>
       </c>
       <c r="I110" t="n">
-        <v>3300</v>
+        <v>731</v>
       </c>
       <c r="J110" t="n">
-        <v>931</v>
-      </c>
-      <c r="K110" t="n">
-        <v>22</v>
+        <v>17.28</v>
       </c>
     </row>
     <row r="111">
@@ -3820,26 +3614,23 @@
         <v>3761</v>
       </c>
       <c r="D111" t="n">
-        <v>3300</v>
+        <v>3960</v>
       </c>
       <c r="E111" t="inlineStr"/>
       <c r="F111" t="n">
         <v>3510</v>
       </c>
       <c r="G111" t="n">
-        <v>3570</v>
+        <v>3500</v>
       </c>
       <c r="H111" t="n">
         <v>3500</v>
       </c>
       <c r="I111" t="n">
-        <v>3300</v>
+        <v>261</v>
       </c>
       <c r="J111" t="n">
-        <v>461</v>
-      </c>
-      <c r="K111" t="n">
-        <v>12.26</v>
+        <v>6.94</v>
       </c>
     </row>
     <row r="112">
@@ -3853,25 +3644,22 @@
         <v>3291</v>
       </c>
       <c r="D112" t="n">
-        <v>3300</v>
+        <v>3960</v>
       </c>
       <c r="E112" t="inlineStr"/>
       <c r="F112" t="n">
-        <v>3323.33</v>
+        <v>3310</v>
       </c>
       <c r="G112" t="n">
-        <v>3370</v>
+        <v>2500</v>
       </c>
       <c r="H112" t="n">
         <v>2500</v>
       </c>
       <c r="I112" t="n">
-        <v>2500</v>
+        <v>791</v>
       </c>
       <c r="J112" t="n">
-        <v>791</v>
-      </c>
-      <c r="K112" t="n">
         <v>24.04</v>
       </c>
     </row>
@@ -3886,25 +3674,22 @@
         <v>3291</v>
       </c>
       <c r="D113" t="n">
-        <v>2800</v>
+        <v>3360</v>
       </c>
       <c r="E113" t="inlineStr"/>
       <c r="F113" t="n">
-        <v>3361.33</v>
+        <v>3310</v>
       </c>
       <c r="G113" t="n">
-        <v>3370</v>
+        <v>2500</v>
       </c>
       <c r="H113" t="n">
         <v>2500</v>
       </c>
       <c r="I113" t="n">
-        <v>2500</v>
+        <v>791</v>
       </c>
       <c r="J113" t="n">
-        <v>791</v>
-      </c>
-      <c r="K113" t="n">
         <v>24.04</v>
       </c>
     </row>
@@ -3927,7 +3712,6 @@
       <c r="H114" t="inlineStr"/>
       <c r="I114" t="inlineStr"/>
       <c r="J114" t="inlineStr"/>
-      <c r="K114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" s="1" t="n"/>
@@ -3943,14 +3727,13 @@
       <c r="E115" t="inlineStr"/>
       <c r="F115" t="inlineStr"/>
       <c r="G115" t="inlineStr"/>
-      <c r="H115" t="inlineStr"/>
+      <c r="H115" t="n">
+        <v>6275</v>
+      </c>
       <c r="I115" t="n">
-        <v>6275</v>
+        <v>0</v>
       </c>
       <c r="J115" t="n">
-        <v>0</v>
-      </c>
-      <c r="K115" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3968,14 +3751,13 @@
       <c r="E116" t="inlineStr"/>
       <c r="F116" t="inlineStr"/>
       <c r="G116" t="inlineStr"/>
-      <c r="H116" t="inlineStr"/>
+      <c r="H116" t="n">
+        <v>5962</v>
+      </c>
       <c r="I116" t="n">
-        <v>5962</v>
+        <v>0</v>
       </c>
       <c r="J116" t="n">
-        <v>0</v>
-      </c>
-      <c r="K116" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3993,14 +3775,13 @@
       <c r="E117" t="inlineStr"/>
       <c r="F117" t="inlineStr"/>
       <c r="G117" t="inlineStr"/>
-      <c r="H117" t="inlineStr"/>
+      <c r="H117" t="n">
+        <v>5648</v>
+      </c>
       <c r="I117" t="n">
-        <v>5648</v>
+        <v>0</v>
       </c>
       <c r="J117" t="n">
-        <v>0</v>
-      </c>
-      <c r="K117" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4018,14 +3799,13 @@
       <c r="E118" t="inlineStr"/>
       <c r="F118" t="inlineStr"/>
       <c r="G118" t="inlineStr"/>
-      <c r="H118" t="inlineStr"/>
+      <c r="H118" t="n">
+        <v>5020</v>
+      </c>
       <c r="I118" t="n">
-        <v>5020</v>
+        <v>0</v>
       </c>
       <c r="J118" t="n">
-        <v>0</v>
-      </c>
-      <c r="K118" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4043,14 +3823,13 @@
       <c r="E119" t="inlineStr"/>
       <c r="F119" t="inlineStr"/>
       <c r="G119" t="inlineStr"/>
-      <c r="H119" t="inlineStr"/>
+      <c r="H119" t="n">
+        <v>4393</v>
+      </c>
       <c r="I119" t="n">
-        <v>4393</v>
+        <v>0</v>
       </c>
       <c r="J119" t="n">
-        <v>0</v>
-      </c>
-      <c r="K119" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4068,14 +3847,13 @@
       <c r="E120" t="inlineStr"/>
       <c r="F120" t="inlineStr"/>
       <c r="G120" t="inlineStr"/>
-      <c r="H120" t="inlineStr"/>
+      <c r="H120" t="n">
+        <v>4393</v>
+      </c>
       <c r="I120" t="n">
-        <v>4393</v>
+        <v>0</v>
       </c>
       <c r="J120" t="n">
-        <v>0</v>
-      </c>
-      <c r="K120" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4108,17 +3886,12 @@
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>Geely Coolray Promo</t>
-        </is>
-      </c>
-      <c r="H121" t="inlineStr">
-        <is>
           <t>Kia Sportage SLS</t>
         </is>
       </c>
+      <c r="H121" t="inlineStr"/>
       <c r="I121" t="inlineStr"/>
       <c r="J121" t="inlineStr"/>
-      <c r="K121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" s="1" t="n"/>
@@ -4131,25 +3904,22 @@
         <v>6275</v>
       </c>
       <c r="D122" t="n">
-        <v>3800</v>
+        <v>4560</v>
       </c>
       <c r="E122" t="inlineStr"/>
       <c r="F122" t="n">
         <v>3500</v>
       </c>
       <c r="G122" t="n">
-        <v>4170</v>
+        <v>3500</v>
       </c>
       <c r="H122" t="n">
         <v>3500</v>
       </c>
       <c r="I122" t="n">
-        <v>3500</v>
+        <v>2775</v>
       </c>
       <c r="J122" t="n">
-        <v>2775</v>
-      </c>
-      <c r="K122" t="n">
         <v>44.22</v>
       </c>
     </row>
@@ -4164,25 +3934,22 @@
         <v>5962</v>
       </c>
       <c r="D123" t="n">
-        <v>3800</v>
+        <v>4560</v>
       </c>
       <c r="E123" t="inlineStr"/>
       <c r="F123" t="n">
         <v>3330</v>
       </c>
       <c r="G123" t="n">
-        <v>3870</v>
+        <v>3500</v>
       </c>
       <c r="H123" t="n">
-        <v>3500</v>
+        <v>3330</v>
       </c>
       <c r="I123" t="n">
-        <v>3330</v>
+        <v>2632</v>
       </c>
       <c r="J123" t="n">
-        <v>2632</v>
-      </c>
-      <c r="K123" t="n">
         <v>44.15</v>
       </c>
     </row>
@@ -4197,25 +3964,22 @@
         <v>5648</v>
       </c>
       <c r="D124" t="n">
-        <v>3300</v>
+        <v>3960</v>
       </c>
       <c r="E124" t="inlineStr"/>
       <c r="F124" t="n">
         <v>3150</v>
       </c>
       <c r="G124" t="n">
-        <v>3570</v>
+        <v>3300</v>
       </c>
       <c r="H124" t="n">
-        <v>3300</v>
+        <v>3150</v>
       </c>
       <c r="I124" t="n">
-        <v>3150</v>
+        <v>2498</v>
       </c>
       <c r="J124" t="n">
-        <v>2498</v>
-      </c>
-      <c r="K124" t="n">
         <v>44.23</v>
       </c>
     </row>
@@ -4230,25 +3994,22 @@
         <v>5020</v>
       </c>
       <c r="D125" t="n">
-        <v>3300</v>
+        <v>3960</v>
       </c>
       <c r="E125" t="inlineStr"/>
       <c r="F125" t="n">
         <v>3150</v>
       </c>
       <c r="G125" t="n">
-        <v>3570</v>
+        <v>3300</v>
       </c>
       <c r="H125" t="n">
-        <v>3300</v>
+        <v>3150</v>
       </c>
       <c r="I125" t="n">
-        <v>3150</v>
+        <v>1870</v>
       </c>
       <c r="J125" t="n">
-        <v>1870</v>
-      </c>
-      <c r="K125" t="n">
         <v>37.25</v>
       </c>
     </row>
@@ -4263,25 +4024,22 @@
         <v>4393</v>
       </c>
       <c r="D126" t="n">
-        <v>3300</v>
+        <v>3960</v>
       </c>
       <c r="E126" t="inlineStr"/>
       <c r="F126" t="n">
         <v>2980</v>
       </c>
       <c r="G126" t="n">
-        <v>3370</v>
+        <v>2500</v>
       </c>
       <c r="H126" t="n">
         <v>2500</v>
       </c>
       <c r="I126" t="n">
-        <v>2500</v>
+        <v>1893</v>
       </c>
       <c r="J126" t="n">
-        <v>1893</v>
-      </c>
-      <c r="K126" t="n">
         <v>43.09</v>
       </c>
     </row>
@@ -4296,25 +4054,22 @@
         <v>4393</v>
       </c>
       <c r="D127" t="n">
-        <v>2800</v>
+        <v>3360</v>
       </c>
       <c r="E127" t="inlineStr"/>
       <c r="F127" t="n">
         <v>2980</v>
       </c>
       <c r="G127" t="n">
-        <v>3370</v>
+        <v>2500</v>
       </c>
       <c r="H127" t="n">
         <v>2500</v>
       </c>
       <c r="I127" t="n">
-        <v>2500</v>
+        <v>1893</v>
       </c>
       <c r="J127" t="n">
-        <v>1893</v>
-      </c>
-      <c r="K127" t="n">
         <v>43.09</v>
       </c>
     </row>
@@ -4341,7 +4096,6 @@
       <c r="H128" t="inlineStr"/>
       <c r="I128" t="inlineStr"/>
       <c r="J128" t="inlineStr"/>
-      <c r="K128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" s="1" t="n"/>
@@ -4357,14 +4111,13 @@
       <c r="E129" t="inlineStr"/>
       <c r="F129" t="inlineStr"/>
       <c r="G129" t="inlineStr"/>
-      <c r="H129" t="inlineStr"/>
+      <c r="H129" t="n">
+        <v>7484</v>
+      </c>
       <c r="I129" t="n">
-        <v>7484</v>
+        <v>0</v>
       </c>
       <c r="J129" t="n">
-        <v>0</v>
-      </c>
-      <c r="K129" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4382,14 +4135,13 @@
       <c r="E130" t="inlineStr"/>
       <c r="F130" t="inlineStr"/>
       <c r="G130" t="inlineStr"/>
-      <c r="H130" t="inlineStr"/>
+      <c r="H130" t="n">
+        <v>7110</v>
+      </c>
       <c r="I130" t="n">
-        <v>7110</v>
+        <v>0</v>
       </c>
       <c r="J130" t="n">
-        <v>0</v>
-      </c>
-      <c r="K130" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4407,14 +4159,13 @@
       <c r="E131" t="inlineStr"/>
       <c r="F131" t="inlineStr"/>
       <c r="G131" t="inlineStr"/>
-      <c r="H131" t="inlineStr"/>
+      <c r="H131" t="n">
+        <v>6736</v>
+      </c>
       <c r="I131" t="n">
-        <v>6736</v>
+        <v>0</v>
       </c>
       <c r="J131" t="n">
-        <v>0</v>
-      </c>
-      <c r="K131" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4432,14 +4183,13 @@
       <c r="E132" t="inlineStr"/>
       <c r="F132" t="inlineStr"/>
       <c r="G132" t="inlineStr"/>
-      <c r="H132" t="inlineStr"/>
+      <c r="H132" t="n">
+        <v>5988</v>
+      </c>
       <c r="I132" t="n">
-        <v>5988</v>
+        <v>0</v>
       </c>
       <c r="J132" t="n">
-        <v>0</v>
-      </c>
-      <c r="K132" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4457,14 +4207,13 @@
       <c r="E133" t="inlineStr"/>
       <c r="F133" t="inlineStr"/>
       <c r="G133" t="inlineStr"/>
-      <c r="H133" t="inlineStr"/>
+      <c r="H133" t="n">
+        <v>5239</v>
+      </c>
       <c r="I133" t="n">
-        <v>5239</v>
+        <v>0</v>
       </c>
       <c r="J133" t="n">
-        <v>0</v>
-      </c>
-      <c r="K133" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4482,14 +4231,13 @@
       <c r="E134" t="inlineStr"/>
       <c r="F134" t="inlineStr"/>
       <c r="G134" t="inlineStr"/>
-      <c r="H134" t="inlineStr"/>
+      <c r="H134" t="n">
+        <v>5239</v>
+      </c>
       <c r="I134" t="n">
-        <v>5239</v>
+        <v>0</v>
       </c>
       <c r="J134" t="n">
-        <v>0</v>
-      </c>
-      <c r="K134" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4516,7 +4264,7 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>Haval F7X / Nissan X-Trail</t>
+          <t>Haval Dargo</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
@@ -4526,17 +4274,12 @@
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>Haval F7 AT</t>
-        </is>
-      </c>
-      <c r="H135" t="inlineStr">
-        <is>
           <t xml:space="preserve">Nissan Xtrail </t>
         </is>
       </c>
+      <c r="H135" t="inlineStr"/>
       <c r="I135" t="inlineStr"/>
       <c r="J135" t="inlineStr"/>
-      <c r="K135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" s="1" t="n"/>
@@ -4549,27 +4292,24 @@
         <v>7484</v>
       </c>
       <c r="D136" t="n">
+        <v>5760</v>
+      </c>
+      <c r="E136" t="n">
+        <v>10472</v>
+      </c>
+      <c r="F136" t="n">
         <v>4800</v>
       </c>
-      <c r="E136" t="n">
-        <v>9100</v>
-      </c>
-      <c r="F136" t="n">
-        <v>4460</v>
-      </c>
       <c r="G136" t="n">
-        <v>4970</v>
+        <v>3900</v>
       </c>
       <c r="H136" t="n">
         <v>3900</v>
       </c>
       <c r="I136" t="n">
-        <v>3900</v>
+        <v>3584</v>
       </c>
       <c r="J136" t="n">
-        <v>3584</v>
-      </c>
-      <c r="K136" t="n">
         <v>47.89</v>
       </c>
     </row>
@@ -4584,27 +4324,24 @@
         <v>7110</v>
       </c>
       <c r="D137" t="n">
-        <v>4800</v>
+        <v>5760</v>
       </c>
       <c r="E137" t="n">
-        <v>8100</v>
+        <v>8726.67</v>
       </c>
       <c r="F137" t="n">
-        <v>4240</v>
+        <v>4560</v>
       </c>
       <c r="G137" t="n">
-        <v>4670</v>
+        <v>3900</v>
       </c>
       <c r="H137" t="n">
         <v>3900</v>
       </c>
       <c r="I137" t="n">
-        <v>3900</v>
+        <v>3210</v>
       </c>
       <c r="J137" t="n">
-        <v>3210</v>
-      </c>
-      <c r="K137" t="n">
         <v>45.15</v>
       </c>
     </row>
@@ -4619,27 +4356,24 @@
         <v>6736</v>
       </c>
       <c r="D138" t="n">
-        <v>4400</v>
+        <v>5280</v>
       </c>
       <c r="E138" t="n">
-        <v>6250</v>
+        <v>7382.86</v>
       </c>
       <c r="F138" t="n">
-        <v>4020</v>
+        <v>4320</v>
       </c>
       <c r="G138" t="n">
-        <v>4270</v>
+        <v>3700</v>
       </c>
       <c r="H138" t="n">
         <v>3700</v>
       </c>
       <c r="I138" t="n">
-        <v>3700</v>
+        <v>3036</v>
       </c>
       <c r="J138" t="n">
-        <v>3036</v>
-      </c>
-      <c r="K138" t="n">
         <v>45.07</v>
       </c>
     </row>
@@ -4654,27 +4388,24 @@
         <v>5988</v>
       </c>
       <c r="D139" t="n">
-        <v>4400</v>
+        <v>5280</v>
       </c>
       <c r="E139" t="n">
-        <v>5500</v>
+        <v>6387.93</v>
       </c>
       <c r="F139" t="n">
-        <v>4020</v>
+        <v>4320</v>
       </c>
       <c r="G139" t="n">
-        <v>4270</v>
+        <v>3700</v>
       </c>
       <c r="H139" t="n">
         <v>3700</v>
       </c>
       <c r="I139" t="n">
-        <v>3700</v>
+        <v>2288</v>
       </c>
       <c r="J139" t="n">
-        <v>2288</v>
-      </c>
-      <c r="K139" t="n">
         <v>38.21</v>
       </c>
     </row>
@@ -4689,27 +4420,24 @@
         <v>5239</v>
       </c>
       <c r="D140" t="n">
-        <v>4400</v>
+        <v>5280</v>
       </c>
       <c r="E140" t="n">
-        <v>5300</v>
+        <v>5759.62</v>
       </c>
       <c r="F140" t="n">
-        <v>3817.62</v>
+        <v>4080</v>
       </c>
       <c r="G140" t="n">
-        <v>3970</v>
+        <v>2700</v>
       </c>
       <c r="H140" t="n">
         <v>2700</v>
       </c>
       <c r="I140" t="n">
-        <v>2700</v>
+        <v>2539</v>
       </c>
       <c r="J140" t="n">
-        <v>2539</v>
-      </c>
-      <c r="K140" t="n">
         <v>48.46</v>
       </c>
     </row>
@@ -4724,27 +4452,24 @@
         <v>5239</v>
       </c>
       <c r="D141" t="n">
-        <v>3900</v>
+        <v>4680</v>
       </c>
       <c r="E141" t="n">
-        <v>4800</v>
+        <v>5550.17</v>
       </c>
       <c r="F141" t="n">
-        <v>3896.33</v>
+        <v>4080</v>
       </c>
       <c r="G141" t="n">
-        <v>3970</v>
+        <v>2700</v>
       </c>
       <c r="H141" t="n">
         <v>2700</v>
       </c>
       <c r="I141" t="n">
-        <v>2700</v>
+        <v>2539</v>
       </c>
       <c r="J141" t="n">
-        <v>2539</v>
-      </c>
-      <c r="K141" t="n">
         <v>48.46</v>
       </c>
     </row>
@@ -4764,22 +4489,21 @@
           <t>Volkswagen Caravelle T6 Di; Hyundai H-1 II rest. 2</t>
         </is>
       </c>
-      <c r="D142" t="inlineStr"/>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>Hyundai Staria</t>
+        </is>
+      </c>
       <c r="E142" t="inlineStr"/>
       <c r="F142" t="inlineStr">
         <is>
           <t>Hyundai H-1 AT</t>
         </is>
       </c>
-      <c r="G142" t="inlineStr">
-        <is>
-          <t>Hyundai Grand Starex AT</t>
-        </is>
-      </c>
+      <c r="G142" t="inlineStr"/>
       <c r="H142" t="inlineStr"/>
       <c r="I142" t="inlineStr"/>
       <c r="J142" t="inlineStr"/>
-      <c r="K142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" s="1" t="n"/>
@@ -4791,22 +4515,21 @@
       <c r="C143" t="n">
         <v>6810</v>
       </c>
-      <c r="D143" t="inlineStr"/>
+      <c r="D143" t="n">
+        <v>11880</v>
+      </c>
       <c r="E143" t="inlineStr"/>
       <c r="F143" t="n">
         <v>8080</v>
       </c>
-      <c r="G143" t="n">
-        <v>11270</v>
-      </c>
-      <c r="H143" t="inlineStr"/>
+      <c r="G143" t="inlineStr"/>
+      <c r="H143" t="n">
+        <v>6810</v>
+      </c>
       <c r="I143" t="n">
-        <v>6810</v>
+        <v>0</v>
       </c>
       <c r="J143" t="n">
-        <v>0</v>
-      </c>
-      <c r="K143" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4820,22 +4543,21 @@
       <c r="C144" t="n">
         <v>6470</v>
       </c>
-      <c r="D144" t="inlineStr"/>
+      <c r="D144" t="n">
+        <v>11880</v>
+      </c>
       <c r="E144" t="inlineStr"/>
       <c r="F144" t="n">
         <v>7390</v>
       </c>
-      <c r="G144" t="n">
-        <v>10570</v>
-      </c>
-      <c r="H144" t="inlineStr"/>
+      <c r="G144" t="inlineStr"/>
+      <c r="H144" t="n">
+        <v>6470</v>
+      </c>
       <c r="I144" t="n">
-        <v>6470</v>
+        <v>0</v>
       </c>
       <c r="J144" t="n">
-        <v>0</v>
-      </c>
-      <c r="K144" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4849,22 +4571,21 @@
       <c r="C145" t="n">
         <v>6129</v>
       </c>
-      <c r="D145" t="inlineStr"/>
+      <c r="D145" t="n">
+        <v>10920</v>
+      </c>
       <c r="E145" t="inlineStr"/>
       <c r="F145" t="n">
         <v>6930</v>
       </c>
-      <c r="G145" t="n">
-        <v>9670</v>
-      </c>
-      <c r="H145" t="inlineStr"/>
+      <c r="G145" t="inlineStr"/>
+      <c r="H145" t="n">
+        <v>6129</v>
+      </c>
       <c r="I145" t="n">
-        <v>6129</v>
+        <v>0</v>
       </c>
       <c r="J145" t="n">
-        <v>0</v>
-      </c>
-      <c r="K145" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4878,22 +4599,21 @@
       <c r="C146" t="n">
         <v>5448</v>
       </c>
-      <c r="D146" t="inlineStr"/>
+      <c r="D146" t="n">
+        <v>10920</v>
+      </c>
       <c r="E146" t="inlineStr"/>
       <c r="F146" t="n">
         <v>6930</v>
       </c>
-      <c r="G146" t="n">
-        <v>9670</v>
-      </c>
-      <c r="H146" t="inlineStr"/>
+      <c r="G146" t="inlineStr"/>
+      <c r="H146" t="n">
+        <v>5448</v>
+      </c>
       <c r="I146" t="n">
-        <v>5448</v>
+        <v>0</v>
       </c>
       <c r="J146" t="n">
-        <v>0</v>
-      </c>
-      <c r="K146" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4907,22 +4627,21 @@
       <c r="C147" t="n">
         <v>4767</v>
       </c>
-      <c r="D147" t="inlineStr"/>
+      <c r="D147" t="n">
+        <v>10920</v>
+      </c>
       <c r="E147" t="inlineStr"/>
       <c r="F147" t="n">
         <v>6460</v>
       </c>
-      <c r="G147" t="n">
-        <v>9070</v>
-      </c>
-      <c r="H147" t="inlineStr"/>
+      <c r="G147" t="inlineStr"/>
+      <c r="H147" t="n">
+        <v>4767</v>
+      </c>
       <c r="I147" t="n">
-        <v>4767</v>
+        <v>0</v>
       </c>
       <c r="J147" t="n">
-        <v>0</v>
-      </c>
-      <c r="K147" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4936,22 +4655,21 @@
       <c r="C148" t="n">
         <v>4767</v>
       </c>
-      <c r="D148" t="inlineStr"/>
+      <c r="D148" t="n">
+        <v>10200</v>
+      </c>
       <c r="E148" t="inlineStr"/>
       <c r="F148" t="n">
         <v>6460</v>
       </c>
-      <c r="G148" t="n">
-        <v>9070</v>
-      </c>
-      <c r="H148" t="inlineStr"/>
+      <c r="G148" t="inlineStr"/>
+      <c r="H148" t="n">
+        <v>4767</v>
+      </c>
       <c r="I148" t="n">
-        <v>4767</v>
+        <v>0</v>
       </c>
       <c r="J148" t="n">
-        <v>0</v>
-      </c>
-      <c r="K148" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4974,7 +4692,6 @@
       <c r="H149" t="inlineStr"/>
       <c r="I149" t="inlineStr"/>
       <c r="J149" t="inlineStr"/>
-      <c r="K149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" s="1" t="n"/>
@@ -4990,14 +4707,13 @@
       <c r="E150" t="inlineStr"/>
       <c r="F150" t="inlineStr"/>
       <c r="G150" t="inlineStr"/>
-      <c r="H150" t="inlineStr"/>
+      <c r="H150" t="n">
+        <v>8512</v>
+      </c>
       <c r="I150" t="n">
-        <v>8512</v>
+        <v>0</v>
       </c>
       <c r="J150" t="n">
-        <v>0</v>
-      </c>
-      <c r="K150" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5015,14 +4731,13 @@
       <c r="E151" t="inlineStr"/>
       <c r="F151" t="inlineStr"/>
       <c r="G151" t="inlineStr"/>
-      <c r="H151" t="inlineStr"/>
+      <c r="H151" t="n">
+        <v>8087</v>
+      </c>
       <c r="I151" t="n">
-        <v>8087</v>
+        <v>0</v>
       </c>
       <c r="J151" t="n">
-        <v>0</v>
-      </c>
-      <c r="K151" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5040,14 +4755,13 @@
       <c r="E152" t="inlineStr"/>
       <c r="F152" t="inlineStr"/>
       <c r="G152" t="inlineStr"/>
-      <c r="H152" t="inlineStr"/>
+      <c r="H152" t="n">
+        <v>7661</v>
+      </c>
       <c r="I152" t="n">
-        <v>7661</v>
+        <v>0</v>
       </c>
       <c r="J152" t="n">
-        <v>0</v>
-      </c>
-      <c r="K152" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5065,14 +4779,13 @@
       <c r="E153" t="inlineStr"/>
       <c r="F153" t="inlineStr"/>
       <c r="G153" t="inlineStr"/>
-      <c r="H153" t="inlineStr"/>
+      <c r="H153" t="n">
+        <v>6810</v>
+      </c>
       <c r="I153" t="n">
-        <v>6810</v>
+        <v>0</v>
       </c>
       <c r="J153" t="n">
-        <v>0</v>
-      </c>
-      <c r="K153" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5090,14 +4803,13 @@
       <c r="E154" t="inlineStr"/>
       <c r="F154" t="inlineStr"/>
       <c r="G154" t="inlineStr"/>
-      <c r="H154" t="inlineStr"/>
+      <c r="H154" t="n">
+        <v>5959</v>
+      </c>
       <c r="I154" t="n">
-        <v>5959</v>
+        <v>0</v>
       </c>
       <c r="J154" t="n">
-        <v>0</v>
-      </c>
-      <c r="K154" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5115,14 +4827,13 @@
       <c r="E155" t="inlineStr"/>
       <c r="F155" t="inlineStr"/>
       <c r="G155" t="inlineStr"/>
-      <c r="H155" t="inlineStr"/>
+      <c r="H155" t="n">
+        <v>5959</v>
+      </c>
       <c r="I155" t="n">
-        <v>5959</v>
+        <v>0</v>
       </c>
       <c r="J155" t="n">
-        <v>0</v>
-      </c>
-      <c r="K155" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>